<commit_message>
18 parameter change change battery mass (#19)
* Battery mass parameter updated

* Update BOM

* Re-run range parametric model

---------

Co-authored-by: Shiam Chuttoo <wssc10@lunet.lboro.ac.uk>
</commit_message>
<xml_diff>
--- a/External Models/BOM/Bill of Materials.xlsx
+++ b/External Models/BOM/Bill of Materials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bt0712\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wssc10\GitHub\Group 5\External Models\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7D63913-2CA6-41CA-8684-E5FBFDF879EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ADC16AC-31FD-4725-AB87-EE83BD1467FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14355" yWindow="0" windowWidth="14445" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM Report" sheetId="1" r:id="rId1"/>
@@ -867,6 +867,27 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -893,27 +914,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -930,10 +930,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1227,22 +1223,22 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I38"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" style="30" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.453125" style="30" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.7265625" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.1796875" style="11" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.5703125" style="13" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" style="13" customWidth="1"/>
-    <col min="9" max="9" width="32.140625" style="13" customWidth="1"/>
-    <col min="10" max="252" width="11.42578125" style="1" customWidth="1"/>
-    <col min="253" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="5" width="13.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.54296875" style="13" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" style="13" customWidth="1"/>
+    <col min="9" max="9" width="32.1796875" style="13" customWidth="1"/>
+    <col min="10" max="252" width="11.453125" style="1" customWidth="1"/>
+    <col min="253" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1253,12 +1249,12 @@
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
     </row>
-    <row r="2" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="53" t="s">
+    <row r="2" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="55"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="62"/>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
@@ -1266,10 +1262,10 @@
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
     </row>
-    <row r="3" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="56"/>
-      <c r="B3" s="57"/>
-      <c r="C3" s="58"/>
+    <row r="3" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="63"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="65"/>
       <c r="D3" s="36" t="s">
         <v>1</v>
       </c>
@@ -1279,7 +1275,7 @@
       <c r="H3" s="9"/>
       <c r="I3" s="9"/>
     </row>
-    <row r="4" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
@@ -1288,7 +1284,7 @@
       </c>
       <c r="D4" s="12"/>
     </row>
-    <row r="5" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>4</v>
       </c>
@@ -1297,7 +1293,7 @@
       </c>
       <c r="D5" s="14"/>
     </row>
-    <row r="6" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>6</v>
       </c>
@@ -1306,7 +1302,7 @@
       </c>
       <c r="D6" s="16"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A7" s="17"/>
       <c r="B7" s="15"/>
       <c r="C7" s="18"/>
@@ -1317,7 +1313,7 @@
       <c r="H7" s="20"/>
       <c r="I7" s="20"/>
     </row>
-    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
         <v>8</v>
       </c>
@@ -1327,7 +1323,7 @@
       <c r="C8" s="22"/>
       <c r="D8" s="23"/>
     </row>
-    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="24" t="s">
         <v>9</v>
       </c>
@@ -1337,28 +1333,28 @@
       </c>
       <c r="C9" s="26">
         <f ca="1">NOW()</f>
-        <v>46156.556311111111</v>
+        <v>46156.881087731483</v>
       </c>
       <c r="D9" s="23"/>
-      <c r="E9" s="61" t="s">
+      <c r="E9" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="61"/>
-      <c r="G9" s="61"/>
-      <c r="H9" s="59" t="s">
+      <c r="F9" s="68"/>
+      <c r="G9" s="68"/>
+      <c r="H9" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="60"/>
-    </row>
-    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I9" s="67"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="21"/>
       <c r="B10" s="27"/>
       <c r="C10" s="28"/>
       <c r="D10" s="23"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
-    </row>
-    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H10" s="67"/>
+      <c r="I10" s="67"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
         <v>12</v>
       </c>
@@ -1367,13 +1363,13 @@
       </c>
       <c r="C11" s="28"/>
       <c r="D11" s="23"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-    </row>
-    <row r="12" spans="1:9" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="H11" s="67"/>
+      <c r="I11" s="67"/>
+    </row>
+    <row r="12" spans="1:9" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="24"/>
     </row>
-    <row r="13" spans="1:9" s="31" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" s="31" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="50" t="s">
         <v>14</v>
       </c>
@@ -1402,49 +1398,49 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:9" s="31" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="66"/>
-      <c r="B14" s="67" t="s">
+    <row r="14" spans="1:9" s="31" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="57"/>
+      <c r="B14" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="67"/>
-      <c r="D14" s="67">
+      <c r="C14" s="58"/>
+      <c r="D14" s="58">
         <v>1</v>
       </c>
-      <c r="E14" s="67">
+      <c r="E14" s="58">
         <f>SUM(E15,E20,E26,E31)</f>
-        <v>10.700000000000001</v>
-      </c>
-      <c r="F14" s="67">
+        <v>10.25</v>
+      </c>
+      <c r="F14" s="58">
         <f>SUM(F15,F20,F26,F31)</f>
         <v>7700</v>
       </c>
-      <c r="G14" s="67"/>
-      <c r="H14" s="67"/>
-      <c r="I14" s="68"/>
-    </row>
-    <row r="15" spans="1:9" s="31" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="62"/>
-      <c r="B15" s="63" t="s">
+      <c r="G14" s="58"/>
+      <c r="H14" s="58"/>
+      <c r="I14" s="59"/>
+    </row>
+    <row r="15" spans="1:9" s="31" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="53"/>
+      <c r="B15" s="54" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63">
+      <c r="C15" s="54"/>
+      <c r="D15" s="54">
         <v>1</v>
       </c>
-      <c r="E15" s="63">
+      <c r="E15" s="54">
         <f>SUM(E16:E19)</f>
         <v>0.91</v>
       </c>
-      <c r="F15" s="63">
+      <c r="F15" s="54">
         <f>SUM(F16:F19)</f>
         <v>2035</v>
       </c>
-      <c r="G15" s="63"/>
-      <c r="H15" s="63"/>
-      <c r="I15" s="64"/>
-    </row>
-    <row r="16" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G15" s="54"/>
+      <c r="H15" s="54"/>
+      <c r="I15" s="55"/>
+    </row>
+    <row r="16" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="44" t="s">
         <v>24</v>
       </c>
@@ -1473,7 +1469,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="47" t="s">
         <v>29</v>
       </c>
@@ -1502,7 +1498,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="39" t="s">
         <v>33</v>
       </c>
@@ -1531,7 +1527,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="47" t="s">
         <v>36</v>
       </c>
@@ -1560,28 +1556,28 @@
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="62"/>
-      <c r="B20" s="65" t="s">
+    <row r="20" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="53"/>
+      <c r="B20" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="63"/>
-      <c r="D20" s="63">
+      <c r="C20" s="54"/>
+      <c r="D20" s="54">
         <v>1</v>
       </c>
-      <c r="E20" s="63">
+      <c r="E20" s="54">
         <f>SUM(E21:E25)</f>
         <v>6.82</v>
       </c>
-      <c r="F20" s="63">
+      <c r="F20" s="54">
         <f>SUM(F21:F25)</f>
         <v>3325</v>
       </c>
-      <c r="G20" s="63"/>
-      <c r="H20" s="63"/>
-      <c r="I20" s="64"/>
-    </row>
-    <row r="21" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="55"/>
+    </row>
+    <row r="21" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="39" t="s">
         <v>41</v>
       </c>
@@ -1610,7 +1606,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="47" t="s">
         <v>46</v>
       </c>
@@ -1639,7 +1635,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="39" t="s">
         <v>49</v>
       </c>
@@ -1668,7 +1664,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="47" t="s">
         <v>52</v>
       </c>
@@ -1697,7 +1693,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="25" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="39" t="s">
         <v>55</v>
       </c>
@@ -1726,28 +1722,28 @@
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="62"/>
-      <c r="B26" s="63" t="s">
+    <row r="26" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="53"/>
+      <c r="B26" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="63"/>
-      <c r="D26" s="63">
+      <c r="C26" s="54"/>
+      <c r="D26" s="54">
         <v>1</v>
       </c>
-      <c r="E26" s="63">
+      <c r="E26" s="54">
         <f>SUM(E27:E30)</f>
         <v>0.49</v>
       </c>
-      <c r="F26" s="63">
+      <c r="F26" s="54">
         <f>SUM(F27:F30)</f>
         <v>1340</v>
       </c>
-      <c r="G26" s="63"/>
-      <c r="H26" s="63"/>
-      <c r="I26" s="64"/>
-    </row>
-    <row r="27" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G26" s="54"/>
+      <c r="H26" s="54"/>
+      <c r="I26" s="55"/>
+    </row>
+    <row r="27" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="47" t="s">
         <v>58</v>
       </c>
@@ -1776,7 +1772,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
         <v>63</v>
       </c>
@@ -1805,7 +1801,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="29" spans="1:9" s="29" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" s="29" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="47" t="s">
         <v>66</v>
       </c>
@@ -1834,7 +1830,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="39" t="s">
         <v>69</v>
       </c>
@@ -1863,28 +1859,28 @@
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="62"/>
-      <c r="B31" s="63" t="s">
+    <row r="31" spans="1:9" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="53"/>
+      <c r="B31" s="54" t="s">
         <v>74</v>
       </c>
-      <c r="C31" s="63"/>
-      <c r="D31" s="63">
+      <c r="C31" s="54"/>
+      <c r="D31" s="54">
         <v>1</v>
       </c>
-      <c r="E31" s="63">
+      <c r="E31" s="54">
         <f>SUM(E32:E35)</f>
-        <v>2.4800000000000004</v>
-      </c>
-      <c r="F31" s="63">
+        <v>2.0299999999999998</v>
+      </c>
+      <c r="F31" s="54">
         <f>SUM(F32:F35)</f>
         <v>1000</v>
       </c>
-      <c r="G31" s="63"/>
-      <c r="H31" s="63"/>
-      <c r="I31" s="64"/>
-    </row>
-    <row r="32" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G31" s="54"/>
+      <c r="H31" s="54"/>
+      <c r="I31" s="55"/>
+    </row>
+    <row r="32" spans="1:9" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="47" t="s">
         <v>72</v>
       </c>
@@ -1898,7 +1894,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="48">
-        <v>1.85</v>
+        <v>1.4</v>
       </c>
       <c r="F32" s="48">
         <v>520</v>
@@ -1913,7 +1909,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="39" t="s">
         <v>77</v>
       </c>
@@ -1942,7 +1938,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="47" t="s">
         <v>81</v>
       </c>
@@ -1971,7 +1967,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="41" t="s">
         <v>85</v>
       </c>
@@ -2000,7 +1996,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36"/>
       <c r="B36"/>
       <c r="C36"/>
@@ -2011,7 +2007,7 @@
       <c r="H36"/>
       <c r="I36"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37"/>
       <c r="B37"/>
       <c r="C37"/>
@@ -2022,7 +2018,7 @@
       <c r="H37"/>
       <c r="I37"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -2046,12 +2042,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4e4d1510-3355-4c87-8117-7dc7019c3145" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="acd71c02-266c-4423-a1b2-5c09bfff8003">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2244,20 +2242,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4e4d1510-3355-4c87-8117-7dc7019c3145" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="acd71c02-266c-4423-a1b2-5c09bfff8003">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55B94B58-C975-41DD-99ED-CB5B8B8D1F42}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68E0AF97-8124-4C42-91D6-ACBDDC39A597}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="4e4d1510-3355-4c87-8117-7dc7019c3145"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="acd71c02-266c-4423-a1b2-5c09bfff8003"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2282,18 +2287,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68E0AF97-8124-4C42-91D6-ACBDDC39A597}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55B94B58-C975-41DD-99ED-CB5B8B8D1F42}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="4e4d1510-3355-4c87-8117-7dc7019c3145"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="acd71c02-266c-4423-a1b2-5c09bfff8003"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>